<commit_message>
[MaxUseTempBenchmark.xlsx]:Removed a stray character in the excel sheet causing errors.
</commit_message>
<xml_diff>
--- a/DataVaryingTemperature/MaxUseTempBenchmark.xlsx
+++ b/DataVaryingTemperature/MaxUseTempBenchmark.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\METALS\DataVaryingTemperature\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9295A3FB-9011-43E6-A0E4-93CE606218B7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C4B1D92B-B3BD-4542-AF4F-68108845B07E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="7170" yWindow="4185" windowWidth="21600" windowHeight="11295" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -23,7 +23,6 @@
     <definedName name="Youngs_Modulus">Reference!$B$3:$D$3</definedName>
   </definedNames>
   <calcPr calcId="191029"/>
-  <fileRecoveryPr repairLoad="1"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
@@ -44,7 +43,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="48" uniqueCount="33">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="47" uniqueCount="32">
   <si>
     <t>Attribute</t>
   </si>
@@ -140,9 +139,6 @@
   </si>
   <si>
     <t>Degree Celsius</t>
-  </si>
-  <si>
-    <t>s</t>
   </si>
 </sst>
 </file>
@@ -532,7 +528,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:N16"/>
+  <dimension ref="A1:M5"/>
   <sheetFormatPr defaultColWidth="9.140625" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="20.7109375" style="1" customWidth="1"/>
@@ -547,7 +543,7 @@
     <col min="700" max="16384" width="9.140625" style="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:14" s="8" customFormat="1" ht="18.75" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:13" s="8" customFormat="1" ht="18.75" x14ac:dyDescent="0.25">
       <c r="B1" s="8" t="s">
         <v>4</v>
       </c>
@@ -585,7 +581,7 @@
         <v>30</v>
       </c>
     </row>
-    <row r="2" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:13" x14ac:dyDescent="0.25">
       <c r="B2" s="1" t="s">
         <v>7</v>
       </c>
@@ -623,7 +619,7 @@
         <v>31</v>
       </c>
     </row>
-    <row r="3" spans="1:14" ht="18.75" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:13" ht="18.75" x14ac:dyDescent="0.25">
       <c r="A3" s="9" t="s">
         <v>14</v>
       </c>
@@ -664,7 +660,7 @@
         <v>1200</v>
       </c>
     </row>
-    <row r="4" spans="1:14" ht="18.75" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:13" ht="18.75" x14ac:dyDescent="0.25">
       <c r="A4" s="8" t="s">
         <v>23</v>
       </c>
@@ -705,7 +701,7 @@
         <v>1200</v>
       </c>
     </row>
-    <row r="5" spans="1:14" ht="18.75" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:13" ht="18.75" x14ac:dyDescent="0.25">
       <c r="A5" s="10" t="s">
         <v>15</v>
       </c>
@@ -744,11 +740,6 @@
       </c>
       <c r="M5" s="1">
         <v>600</v>
-      </c>
-    </row>
-    <row r="16" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="N16" s="1" t="s">
-        <v>32</v>
       </c>
     </row>
   </sheetData>

</xml_diff>